<commit_message>
Release 3.0.22: update FSales installer
</commit_message>
<xml_diff>
--- a/bao_gia_mau.xlsx
+++ b/bao_gia_mau.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Fsales_PCCC\dist\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Fsales_PCCC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBB976C1-6C9B-4B12-8433-2D34C3C391B7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3810FD16-5A8A-4A3A-B3E5-6C89323B2F88}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="13170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -145,13 +145,13 @@
     <t>- Giao hàng tại kho của bên bán tại Khu công nghiệp Từ Liêm, Bắc Từ Liêm, Hà Nội.</t>
   </si>
   <si>
-    <t>* Tài khoản thanh toán Cá nhân: 19020916593016</t>
-  </si>
-  <si>
     <t>- Tại ngân hàng Techcombank</t>
   </si>
   <si>
-    <t>- CTK:  Phí Ngọc Tùng</t>
+    <t>* Tài khoản thanh toán số: 11488686</t>
+  </si>
+  <si>
+    <t>- CTK:  Công ty CP dịch vụ kỹ thuật PCCC Việt Nam</t>
   </si>
 </sst>
 </file>
@@ -4126,7 +4126,7 @@
     <row r="102" spans="1:25" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="23"/>
       <c r="B102" s="84" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C102" s="67"/>
       <c r="D102" s="67"/>
@@ -4155,7 +4155,7 @@
     <row r="103" spans="1:25" s="34" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="58"/>
       <c r="B103" s="85" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C103" s="69"/>
       <c r="D103" s="69"/>

</xml_diff>